<commit_message>
docs: el resumen ejecutivo y el Excel corrigen el porqué del suelo de alarmas
Retirada la atribución "resolución corregida más deriva de 2,6x", que contaba
las puntuaciones consecutivas como independientes. Sustituida por el límite de
representabilidad: con ventanas solapadas al 75 %, una recalibración de 236
puntuaciones contiene 59 observaciones efectivas, y con 7 controles estadísticos
el alpha mínimo representable es 7/59 = 0,119.

Por debajo de ese valor la petición no es representable y el gate entrega su
suelo de 0,083 se pida lo que se pida. El suelo pasa a ser consecuencia del
tamaño de la muestra, y es la razón estructural para declarar el presupuesto
medido en vez de prometer uno nominal.

El suelo, la curva de operación y la correlación entre alertas no se tocan.
Ambos documentos llevan el aviso de corrección citando challenge y respuesta.

Código en codex/dq-monitor-trim-3sigma (ce33b87).

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/reports/dq_entregables/resultados_dq.xlsx
+++ b/results/reports/dq_entregables/resultados_dq.xlsx
@@ -985,7 +985,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1158,16 +1158,24 @@
     <row r="13" ht="46" customHeight="1">
       <c r="A13" s="11" t="inlineStr">
         <is>
-          <t>El exceso sobre el nominal tiene dos causas medidas. La resolución de la muestra de calibración ya está corregida ampliando la ventana. La que queda es deriva: cada control realiza ~2,6 veces su tasa nominal porque el tramo reciente no predice la cola del siguiente. Esa es la que fija el suelo y no se arregla repartiendo mejor.</t>
+          <t>POR QUÉ EXISTE EL SUELO: las ventanas de 20 sesiones con paso 5 solapan al 75 %, así que una recalibración de 236 puntuaciones contiene solo 59 observaciones EFECTIVAS. Con 7 controles estadísticos, el α más pequeño que esa muestra puede representar es 7/59 = 0.119. Por debajo, la petición no es representable: el umbral cae en el máximo empírico y el gate entrega su suelo. El suelo es consecuencia del tamaño de la muestra, no una curiosidad.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="46" customHeight="1">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>CORRECCIÓN REGISTRADA: una versión anterior atribuía el exceso a «resolución corregida más deriva de 2,6x». Esa atribución contaba las puntuaciones consecutivas como independientes y queda RETIRADA. El suelo y la curva no se ven afectados: son observaciones, no atribuciones causales.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A11:E11"/>
+  <mergeCells count="5">
     <mergeCell ref="A12:E12"/>
     <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A11:E11"/>
     <mergeCell ref="A13:E13"/>
+    <mergeCell ref="A14:E14"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>